<commit_message>
changed "iifvg*" files into "i2fvg*"; updated the cols_dicts; created the financial pipeline; updated the readme
</commit_message>
<xml_diff>
--- a/cols_dict.xlsx
+++ b/cols_dict.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vesnic\OneDrive - Area Science Park\Documenti\GitLab\imprese-fvg\script\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://areasciencepark.sharepoint.com/sites/InnovationIntelligence/Documenti condivisi/Evoluzione I2/FAIR/script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7CD2F2A-A51A-47D0-AACB-7A4D55080AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{B7CD2F2A-A51A-47D0-AACB-7A4D55080AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4ABB3C3-B36C-40C8-A5AD-4E4E800C9FD8}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-13068" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="anagrafica" sheetId="1" r:id="rId1"/>
@@ -346,9 +346,6 @@
     <t>ordine_INSIEL</t>
   </si>
   <si>
-    <t>ordine_iifvg</t>
-  </si>
-  <si>
     <t>fonte</t>
   </si>
   <si>
@@ -414,13 +411,16 @@
   <si>
     <t>Impresa
 Ultima Modifica</t>
+  </si>
+  <si>
+    <t>ordine_i2fvg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -459,6 +459,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -583,16 +591,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -605,25 +612,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -638,20 +642,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -663,7 +664,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -674,24 +675,28 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -974,7 +979,7 @@
     <tableColumn id="2" xr3:uid="{314D2832-223B-4CB1-A27E-35B056DD8234}" name="nomi_colonne_corretti" dataDxfId="12"/>
     <tableColumn id="6" xr3:uid="{C33E96E5-556B-4AC3-A402-347B787E7E6B}" name="nomi_colonne_export" dataDxfId="11"/>
     <tableColumn id="3" xr3:uid="{F2FD8189-7CD5-447E-B456-D2A358625E37}" name="ordine_repo" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{554A28B1-F0E7-4349-84A4-23CD923A87A6}" name="ordine_iifvg" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{554A28B1-F0E7-4349-84A4-23CD923A87A6}" name="ordine_i2fvg" dataDxfId="9"/>
     <tableColumn id="5" xr3:uid="{D3517C70-E2A8-4650-8B5E-E772A0A7D5A1}" name="ordine_INSIEL" dataDxfId="8"/>
     <tableColumn id="7" xr3:uid="{5F04E795-40EA-4262-83F5-0EF7160042B2}" name="ordine_AINDO" dataDxfId="7"/>
   </tableColumns>
@@ -989,7 +994,7 @@
     <tableColumn id="1" xr3:uid="{C5021392-6187-4B59-A286-D58A36656049}" name="nomi_colonne_originali" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{BFDA8532-1586-4DDC-9EF0-6F888384F144}" name="nomi_colonne_corretti" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{0E12423C-F1FC-48A1-AF86-9AF23E6F89B7}" name="ordine_repo" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{F8E399BD-2D17-44A3-B60A-5CCFADC05B5C}" name="ordine_iifvg" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{F8E399BD-2D17-44A3-B60A-5CCFADC05B5C}" name="ordine_i2fvg" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{824D4A1A-8F56-460C-B679-459087AC3A87}" name="ordine_INSIEL" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1284,1289 +1289,1289 @@
   <dimension ref="A1:G60"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.36328125" style="14" customWidth="1"/>
-    <col min="2" max="3" width="29.36328125" style="15" customWidth="1"/>
-    <col min="4" max="6" width="29.36328125" style="19" customWidth="1"/>
+    <col min="1" max="1" width="29.36328125" style="12" customWidth="1"/>
+    <col min="2" max="3" width="29.36328125" style="13" customWidth="1"/>
+    <col min="4" max="6" width="29.36328125" style="17" customWidth="1"/>
     <col min="7" max="7" width="20.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D1" s="8" t="s">
+      <c r="C1" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="F1" s="9" t="s">
+      <c r="E1" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G1" s="8" t="s">
-        <v>120</v>
+      <c r="G1" s="7" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="16">
+      <c r="D2" s="14">
         <v>13</v>
       </c>
-      <c r="E2" s="16">
+      <c r="E2" s="14">
         <v>1</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="18">
         <v>1</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="14">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="14">
         <v>34</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="14">
         <v>2</v>
       </c>
-      <c r="F3" s="21">
+      <c r="F3" s="14">
         <v>2</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="14">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="14">
         <v>15</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="14">
         <v>3</v>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="18">
         <v>3</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="17"/>
-      <c r="E5" s="16">
+      <c r="D5" s="15"/>
+      <c r="E5" s="14">
         <v>4</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="14">
         <v>4</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="14">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="14">
         <v>31</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="14">
         <v>5</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="18">
         <v>5</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="14">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="14">
         <v>16</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="14">
         <v>6</v>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="14">
         <v>6</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="14">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="14">
         <v>18</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="14">
         <v>7</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="18">
         <v>7</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="14">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="14">
         <v>23</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="14">
         <v>8</v>
       </c>
-      <c r="F9" s="21">
+      <c r="F9" s="14">
         <v>8</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="14">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="14">
         <v>22</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="14">
         <v>9</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="18">
         <v>9</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="14">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="14">
         <v>21</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="14">
         <v>10</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="14">
         <v>10</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="14">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="14">
         <v>112</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="14">
         <v>11</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="18">
         <v>11</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="14">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="14">
         <v>113</v>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="14">
         <v>12</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="14">
         <v>12</v>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="14">
         <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="14">
         <v>114</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="14">
         <v>13</v>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="18">
         <v>13</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="14">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="14">
         <v>115</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="14">
         <v>14</v>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="14">
         <v>14</v>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="14">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="14">
         <v>116</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="14">
         <v>15</v>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="18">
         <v>15</v>
       </c>
-      <c r="G16" s="17"/>
+      <c r="G16" s="37"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="14">
         <v>117</v>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="14">
         <v>16</v>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="14">
         <v>16</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="14">
         <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="B18" s="11" t="s">
+      <c r="A18" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="16">
+      <c r="D18" s="14">
         <v>118</v>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="14">
         <v>17</v>
       </c>
-      <c r="F18" s="20">
+      <c r="F18" s="18">
         <v>17</v>
       </c>
-      <c r="G18" s="17"/>
+      <c r="G18" s="15"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D19" s="16">
+      <c r="D19" s="14">
         <v>119</v>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="14">
         <v>18</v>
       </c>
-      <c r="F19" s="21">
+      <c r="F19" s="14">
         <v>18</v>
       </c>
-      <c r="G19" s="16">
+      <c r="G19" s="14">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="16">
+      <c r="D20" s="14">
         <v>120</v>
       </c>
-      <c r="E20" s="16">
+      <c r="E20" s="14">
         <v>19</v>
       </c>
-      <c r="F20" s="20">
+      <c r="F20" s="18">
         <v>19</v>
       </c>
-      <c r="G20" s="16">
+      <c r="G20" s="14">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="16">
+      <c r="D21" s="14">
         <v>12</v>
       </c>
-      <c r="E21" s="16">
+      <c r="E21" s="14">
         <v>20</v>
       </c>
-      <c r="F21" s="21">
+      <c r="F21" s="14">
         <v>20</v>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="14">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="14">
         <v>33</v>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="14">
         <v>21</v>
       </c>
-      <c r="F22" s="20">
+      <c r="F22" s="18">
         <v>21</v>
       </c>
-      <c r="G22" s="16">
+      <c r="G22" s="14">
         <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="17"/>
-      <c r="E23" s="16">
+      <c r="D23" s="15"/>
+      <c r="E23" s="14">
         <v>22</v>
       </c>
-      <c r="F23" s="21">
+      <c r="F23" s="14">
         <v>22</v>
       </c>
-      <c r="G23" s="16">
+      <c r="G23" s="14">
         <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D24" s="17"/>
-      <c r="E24" s="16">
+      <c r="D24" s="15"/>
+      <c r="E24" s="14">
         <v>23</v>
       </c>
-      <c r="F24" s="20">
+      <c r="F24" s="18">
         <v>23</v>
       </c>
-      <c r="G24" s="16">
+      <c r="G24" s="14">
         <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="16">
+      <c r="D25" s="14">
         <v>32</v>
       </c>
-      <c r="E25" s="16">
+      <c r="E25" s="14">
         <v>24</v>
       </c>
-      <c r="F25" s="21">
+      <c r="F25" s="14">
         <v>24</v>
       </c>
-      <c r="G25" s="16">
+      <c r="G25" s="14">
         <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D26" s="17"/>
-      <c r="E26" s="16">
+      <c r="D26" s="15"/>
+      <c r="E26" s="14">
         <v>25</v>
       </c>
-      <c r="F26" s="20">
+      <c r="F26" s="18">
         <v>25</v>
       </c>
-      <c r="G26" s="16">
+      <c r="G26" s="14">
         <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="17"/>
-      <c r="E27" s="16">
+      <c r="D27" s="15"/>
+      <c r="E27" s="14">
         <v>26</v>
       </c>
-      <c r="F27" s="21">
+      <c r="F27" s="14">
         <v>26</v>
       </c>
-      <c r="G27" s="16">
+      <c r="G27" s="14">
         <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="16">
+      <c r="D28" s="14">
         <v>72</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E28" s="14">
         <v>27</v>
       </c>
-      <c r="F28" s="20">
+      <c r="F28" s="18">
         <v>27</v>
       </c>
-      <c r="G28" s="16">
+      <c r="G28" s="14">
         <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="16">
+      <c r="D29" s="14">
         <v>73</v>
       </c>
-      <c r="E29" s="16">
+      <c r="E29" s="14">
         <v>28</v>
       </c>
-      <c r="F29" s="21">
+      <c r="F29" s="14">
         <v>28</v>
       </c>
-      <c r="G29" s="16">
+      <c r="G29" s="14">
         <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
+      <c r="A30" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="14">
         <v>74</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="14">
         <v>29</v>
       </c>
-      <c r="F30" s="20">
+      <c r="F30" s="18">
         <v>29</v>
       </c>
-      <c r="G30" s="16">
+      <c r="G30" s="14">
         <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="10" t="s">
+      <c r="A31" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="14">
         <v>14</v>
       </c>
-      <c r="E31" s="16">
+      <c r="E31" s="14">
         <v>30</v>
       </c>
-      <c r="F31" s="21">
+      <c r="F31" s="14">
         <v>30</v>
       </c>
-      <c r="G31" s="16">
+      <c r="G31" s="14">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D32" s="17"/>
-      <c r="E32" s="16">
+      <c r="D32" s="15"/>
+      <c r="E32" s="14">
         <v>31</v>
       </c>
-      <c r="F32" s="20">
+      <c r="F32" s="18">
         <v>31</v>
       </c>
-      <c r="G32" s="17"/>
+      <c r="G32" s="15"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="10" t="s">
+      <c r="A33" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="C33" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D33" s="16">
+      <c r="D33" s="14">
         <v>39</v>
       </c>
-      <c r="E33" s="16">
+      <c r="E33" s="14">
         <v>32</v>
       </c>
-      <c r="F33" s="21">
+      <c r="F33" s="14">
         <v>32</v>
       </c>
-      <c r="G33" s="16">
+      <c r="G33" s="14">
         <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="10" t="s">
+      <c r="A34" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D34" s="16">
+      <c r="D34" s="14">
         <v>46</v>
       </c>
-      <c r="E34" s="16">
+      <c r="E34" s="14">
         <v>33</v>
       </c>
-      <c r="F34" s="20">
+      <c r="F34" s="18">
         <v>33</v>
       </c>
-      <c r="G34" s="16">
+      <c r="G34" s="14">
         <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C35" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="16">
+      <c r="D35" s="14">
         <v>40</v>
       </c>
-      <c r="E35" s="16">
+      <c r="E35" s="14">
         <v>34</v>
       </c>
-      <c r="F35" s="21">
+      <c r="F35" s="14">
         <v>34</v>
       </c>
-      <c r="G35" s="16">
+      <c r="G35" s="14">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D36" s="16">
+      <c r="D36" s="14">
         <v>26</v>
       </c>
-      <c r="E36" s="16">
+      <c r="E36" s="14">
         <v>35</v>
       </c>
-      <c r="F36" s="20">
+      <c r="F36" s="18">
         <v>35</v>
       </c>
-      <c r="G36" s="16">
+      <c r="G36" s="14">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" s="10" t="s">
+      <c r="A37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D37" s="17"/>
-      <c r="E37" s="16">
+      <c r="D37" s="15"/>
+      <c r="E37" s="14">
         <v>36</v>
       </c>
-      <c r="F37" s="21">
+      <c r="F37" s="14">
         <v>36</v>
       </c>
-      <c r="G37" s="17"/>
+      <c r="G37" s="15"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" s="10" t="s">
+      <c r="A38" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="17"/>
-      <c r="E38" s="16">
+      <c r="D38" s="15"/>
+      <c r="E38" s="14">
         <v>37</v>
       </c>
-      <c r="F38" s="20">
+      <c r="F38" s="18">
         <v>37</v>
       </c>
-      <c r="G38" s="17"/>
+      <c r="G38" s="15"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
+      <c r="A39" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C39" s="11" t="s">
+      <c r="C39" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="D39" s="17"/>
-      <c r="E39" s="16">
+      <c r="D39" s="15"/>
+      <c r="E39" s="14">
         <v>38</v>
       </c>
-      <c r="F39" s="21">
+      <c r="F39" s="14">
         <v>38</v>
       </c>
-      <c r="G39" s="17"/>
+      <c r="G39" s="15"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A40" s="10" t="s">
+      <c r="A40" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D40" s="17"/>
-      <c r="E40" s="16">
+      <c r="D40" s="15"/>
+      <c r="E40" s="14">
         <v>39</v>
       </c>
-      <c r="F40" s="20">
+      <c r="F40" s="18">
         <v>39</v>
       </c>
-      <c r="G40" s="17"/>
+      <c r="G40" s="15"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" s="10" t="s">
+      <c r="A41" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C41" s="11" t="s">
+      <c r="C41" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D41" s="17"/>
-      <c r="E41" s="16">
+      <c r="D41" s="15"/>
+      <c r="E41" s="14">
         <v>40</v>
       </c>
-      <c r="F41" s="21">
+      <c r="F41" s="14">
         <v>40</v>
       </c>
-      <c r="G41" s="17"/>
+      <c r="G41" s="15"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="B42" s="11" t="s">
+      <c r="A42" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B42" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="D42" s="16">
+      <c r="D42" s="14">
         <v>42</v>
       </c>
-      <c r="E42" s="16">
+      <c r="E42" s="14">
         <v>41</v>
       </c>
-      <c r="F42" s="20">
+      <c r="F42" s="18">
         <v>41</v>
       </c>
-      <c r="G42" s="16">
+      <c r="G42" s="14">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B43" s="11" t="s">
+      <c r="A43" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C43" s="11" t="s">
+      <c r="C43" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="D43" s="16">
+      <c r="D43" s="14">
         <v>43</v>
       </c>
-      <c r="E43" s="16">
+      <c r="E43" s="14">
         <v>42</v>
       </c>
-      <c r="F43" s="21">
+      <c r="F43" s="14">
         <v>42</v>
       </c>
-      <c r="G43" s="16">
+      <c r="G43" s="14">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="B44" s="11" t="s">
+      <c r="A44" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B44" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C44" s="11" t="s">
+      <c r="C44" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D44" s="16">
+      <c r="D44" s="14">
         <v>44</v>
       </c>
-      <c r="E44" s="16">
+      <c r="E44" s="14">
         <v>43</v>
       </c>
-      <c r="F44" s="20">
+      <c r="F44" s="18">
         <v>43</v>
       </c>
-      <c r="G44" s="16">
+      <c r="G44" s="14">
         <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B45" s="11" t="s">
+      <c r="A45" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B45" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="C45" s="11" t="s">
+      <c r="C45" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="D45" s="16">
+      <c r="D45" s="14">
         <v>45</v>
       </c>
-      <c r="E45" s="16">
+      <c r="E45" s="14">
         <v>44</v>
       </c>
-      <c r="F45" s="21">
+      <c r="F45" s="14">
         <v>44</v>
       </c>
-      <c r="G45" s="16">
+      <c r="G45" s="14">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B46" s="11" t="s">
+      <c r="A46" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B46" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="D46" s="16">
+      <c r="D46" s="14">
         <v>46</v>
       </c>
-      <c r="E46" s="16">
+      <c r="E46" s="14">
         <v>45</v>
       </c>
-      <c r="F46" s="20">
+      <c r="F46" s="18">
         <v>45</v>
       </c>
-      <c r="G46" s="16">
+      <c r="G46" s="14">
         <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B47" s="11" t="s">
+      <c r="A47" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B47" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="C47" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="D47" s="16">
+      <c r="D47" s="14">
         <v>47</v>
       </c>
-      <c r="E47" s="16">
+      <c r="E47" s="14">
         <v>46</v>
       </c>
-      <c r="F47" s="21">
+      <c r="F47" s="14">
         <v>46</v>
       </c>
-      <c r="G47" s="16">
+      <c r="G47" s="14">
         <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="B48" s="11" t="s">
+      <c r="A48" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B48" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C48" s="11" t="s">
+      <c r="C48" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="D48" s="16">
+      <c r="D48" s="14">
         <v>48</v>
       </c>
-      <c r="E48" s="16">
+      <c r="E48" s="14">
         <v>47</v>
       </c>
-      <c r="F48" s="20">
+      <c r="F48" s="18">
         <v>47</v>
       </c>
-      <c r="G48" s="16">
+      <c r="G48" s="14">
         <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" s="10" t="s">
+      <c r="A49" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B49" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="C49" s="11" t="s">
+      <c r="B49" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C49" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D49" s="17"/>
-      <c r="E49" s="16">
+      <c r="D49" s="15"/>
+      <c r="E49" s="14">
         <v>48</v>
       </c>
-      <c r="F49" s="21">
+      <c r="F49" s="14">
         <v>48</v>
       </c>
-      <c r="G49" s="17"/>
+      <c r="G49" s="15"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" s="10" t="s">
+      <c r="A50" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C50" s="11" t="s">
+      <c r="C50" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D50" s="16">
+      <c r="D50" s="14">
         <v>122</v>
       </c>
-      <c r="E50" s="16">
+      <c r="E50" s="14">
         <v>49</v>
       </c>
-      <c r="F50" s="20">
+      <c r="F50" s="18">
         <v>49</v>
       </c>
-      <c r="G50" s="16">
+      <c r="G50" s="14">
         <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" s="10" t="s">
+      <c r="A51" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="B51" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C51" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D51" s="16">
+      <c r="D51" s="14">
         <v>121</v>
       </c>
-      <c r="E51" s="16">
+      <c r="E51" s="14">
         <v>50</v>
       </c>
-      <c r="F51" s="21">
+      <c r="F51" s="14">
         <v>50</v>
       </c>
-      <c r="G51" s="16">
+      <c r="G51" s="14">
         <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" s="12" t="s">
+      <c r="A52" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B52" s="13" t="s">
+      <c r="B52" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="C52" s="13" t="s">
+      <c r="C52" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D52" s="18">
+      <c r="D52" s="16">
         <v>48</v>
       </c>
-      <c r="E52" s="16">
+      <c r="E52" s="14">
         <v>51</v>
       </c>
-      <c r="F52" s="20">
+      <c r="F52" s="18">
         <v>51</v>
       </c>
-      <c r="G52" s="17"/>
+      <c r="G52" s="15"/>
     </row>
     <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A53" s="36" t="s">
-        <v>126</v>
-      </c>
-      <c r="B53" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="C53" s="39" t="s">
-        <v>121</v>
-      </c>
-      <c r="D53" s="16">
+      <c r="A53" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C53" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="D53" s="14">
         <v>140</v>
       </c>
-      <c r="E53" s="37"/>
-      <c r="F53" s="38"/>
-      <c r="G53" s="7"/>
+      <c r="E53" s="34"/>
+      <c r="F53" s="35"/>
+      <c r="G53" s="6"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A54" s="10" t="s">
+      <c r="A54" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B54" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B54" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C54" s="39" t="s">
-        <v>123</v>
-      </c>
-      <c r="D54" s="16">
+      <c r="C54" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="D54" s="14">
         <v>141</v>
       </c>
-      <c r="E54" s="37"/>
-      <c r="F54" s="38"/>
-      <c r="G54" s="7"/>
+      <c r="E54" s="34"/>
+      <c r="F54" s="35"/>
+      <c r="G54" s="6"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A55" s="10" t="s">
+      <c r="A55" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B55" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B55" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="C55" s="39" t="s">
-        <v>125</v>
-      </c>
-      <c r="D55" s="16">
+      <c r="C55" s="36" t="s">
+        <v>124</v>
+      </c>
+      <c r="D55" s="14">
         <v>142</v>
       </c>
-      <c r="E55" s="37"/>
-      <c r="F55" s="38"/>
-      <c r="G55" s="7"/>
+      <c r="E55" s="34"/>
+      <c r="F55" s="35"/>
+      <c r="G55" s="6"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A56" s="26"/>
-      <c r="B56" s="24" t="s">
-        <v>105</v>
-      </c>
-      <c r="C56" s="24" t="s">
-        <v>105</v>
-      </c>
-      <c r="D56" s="25">
+      <c r="A56" s="23"/>
+      <c r="B56" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="C56" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="D56" s="22">
         <v>1</v>
       </c>
-      <c r="E56" s="27"/>
-      <c r="F56" s="27"/>
-      <c r="G56" s="7"/>
+      <c r="E56" s="24"/>
+      <c r="F56" s="24"/>
+      <c r="G56" s="6"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A57" s="26"/>
-      <c r="B57" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="C57" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="D57" s="25">
+      <c r="A57" s="23"/>
+      <c r="B57" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C57" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="D57" s="22">
         <v>2</v>
       </c>
-      <c r="E57" s="27"/>
-      <c r="F57" s="27"/>
-      <c r="G57" s="7"/>
+      <c r="E57" s="24"/>
+      <c r="F57" s="24"/>
+      <c r="G57" s="6"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A58" s="28"/>
-      <c r="B58" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="C58" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="D58" s="29">
+      <c r="A58" s="25"/>
+      <c r="B58" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="C58" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D58" s="26">
         <v>6</v>
       </c>
-      <c r="E58" s="30"/>
-      <c r="F58" s="30"/>
-      <c r="G58" s="7"/>
+      <c r="E58" s="27"/>
+      <c r="F58" s="27"/>
+      <c r="G58" s="6"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A59" s="28"/>
-      <c r="B59" s="24" t="s">
-        <v>108</v>
-      </c>
-      <c r="C59" s="24" t="s">
-        <v>108</v>
-      </c>
-      <c r="D59" s="29">
+      <c r="A59" s="25"/>
+      <c r="B59" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="C59" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="D59" s="26">
         <v>7</v>
       </c>
-      <c r="E59" s="30"/>
-      <c r="F59" s="30"/>
-      <c r="G59" s="7"/>
+      <c r="E59" s="27"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="6"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A60" s="33"/>
-      <c r="B60" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="C60" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="D60" s="35">
+      <c r="A60" s="30"/>
+      <c r="B60" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="C60" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="D60" s="32">
         <v>8</v>
       </c>
-      <c r="E60" s="31"/>
-      <c r="F60" s="32"/>
-      <c r="G60" s="7"/>
+      <c r="E60" s="28"/>
+      <c r="F60" s="29"/>
+      <c r="G60" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2579,31 +2584,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EC41180-559B-4675-B163-F8D668B5C63C}">
-  <dimension ref="A1:XFC12"/>
+  <dimension ref="A1:XFC18"/>
   <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.6328125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21.6328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.54296875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="19.08984375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21.90625" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="9.08984375" style="2"/>
+    <col min="1" max="1" width="22.6328125" customWidth="1"/>
+    <col min="2" max="2" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.54296875" customWidth="1"/>
+    <col min="4" max="4" width="19.08984375" customWidth="1"/>
+    <col min="5" max="5" width="21.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="E1" s="22" t="s">
+      <c r="D1" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="E1" s="19" t="s">
         <v>103</v>
       </c>
       <c r="G1" s="1"/>
@@ -10797,159 +10801,162 @@
       <c r="XFC1" s="1"/>
     </row>
     <row r="2" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="2">
+      <c r="C3" s="20"/>
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3" s="23"/>
+      <c r="E3" s="20"/>
     </row>
     <row r="4" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="2">
+      <c r="C4" s="20"/>
+      <c r="D4">
         <v>3</v>
       </c>
-      <c r="E4" s="23"/>
+      <c r="E4" s="20"/>
     </row>
     <row r="5" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>95</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5">
         <v>4</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5">
         <v>4</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6">
         <v>5</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7">
         <v>6</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7">
         <v>6</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>98</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8">
         <v>7</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8">
         <v>7</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A9" s="26"/>
-      <c r="B9" s="24" t="s">
-        <v>105</v>
-      </c>
-      <c r="C9" s="25">
+      <c r="A9" s="23"/>
+      <c r="B9" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="22">
         <v>-4</v>
       </c>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
     </row>
     <row r="10" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A10" s="26"/>
-      <c r="B10" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="25">
+      <c r="A10" s="23"/>
+      <c r="B10" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="22">
         <v>-3</v>
       </c>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
     </row>
     <row r="11" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A11" s="28"/>
-      <c r="B11" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" s="29">
+      <c r="A11" s="25"/>
+      <c r="B11" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="26">
         <v>-2</v>
       </c>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
     </row>
     <row r="12" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A12" s="28"/>
-      <c r="B12" s="24" t="s">
-        <v>108</v>
-      </c>
-      <c r="C12" s="29">
+      <c r="A12" s="25"/>
+      <c r="B12" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" s="26">
         <v>-1</v>
       </c>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E18" s="38"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10961,26 +10968,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="68cb2d5c-a581-419c-ba44-a83686d3d7f3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="caa3a5b7-d789-4b2e-8526-7e2c3c4e4177" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005FAEDE985A08184DA3C66A029CB09EFC" ma:contentTypeVersion="16" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="7360e2010d99e1044ea4290e6831b202">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="68cb2d5c-a581-419c-ba44-a83686d3d7f3" xmlns:ns3="caa3a5b7-d789-4b2e-8526-7e2c3c4e4177" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6b8f38cda5a3a49459d9615b44dda0f9" ns2:_="" ns3:_="">
     <xsd:import namespace="68cb2d5c-a581-419c-ba44-a83686d3d7f3"/>
@@ -11217,19 +11204,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="68cb2d5c-a581-419c-ba44-a83686d3d7f3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="caa3a5b7-d789-4b2e-8526-7e2c3c4e4177" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB97C882-F295-4EF2-90DB-DCBFFB55BE71}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4094048-0D84-4D7A-940F-9F42F107316C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="bc7534d7-dfa9-4174-b547-ed1d9ab2a704"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="4e4d3f74-de77-4e69-aa0e-048b2a3ea68f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="68cb2d5c-a581-419c-ba44-a83686d3d7f3"/>
+    <ds:schemaRef ds:uri="caa3a5b7-d789-4b2e-8526-7e2c3c4e4177"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11243,5 +11252,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4094048-0D84-4D7A-940F-9F42F107316C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB97C882-F295-4EF2-90DB-DCBFFB55BE71}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="bc7534d7-dfa9-4174-b547-ed1d9ab2a704"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="4e4d3f74-de77-4e69-aa0e-048b2a3ea68f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="68cb2d5c-a581-419c-ba44-a83686d3d7f3"/>
+    <ds:schemaRef ds:uri="caa3a5b7-d789-4b2e-8526-7e2c3c4e4177"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>